<commit_message>
spliting the heuristics and implementing a new heuristic
</commit_message>
<xml_diff>
--- a/Benchmark/UrlManual.xlsx
+++ b/Benchmark/UrlManual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javi2\OneDrive\Documentos\Paper2RO\Benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8C022D-1A7B-4D8F-A168-8B8BCF82A9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C465320-77EE-4205-B7C3-BC4C6C35A1C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-45" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{1722B15F-9DAC-4C50-870B-2F1594AC188D}"/>
+    <workbookView xWindow="-45" yWindow="16080" windowWidth="29040" windowHeight="16440" xr2:uid="{1722B15F-9DAC-4C50-870B-2F1594AC188D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="283">
   <si>
     <t>PDF</t>
   </si>
@@ -684,13 +684,217 @@
   </si>
   <si>
     <t>No accesible</t>
+  </si>
+  <si>
+    <t>2311.02709v1.pdf</t>
+  </si>
+  <si>
+    <t>https://github.com/facebookresearch/detectron2</t>
+  </si>
+  <si>
+    <t>2405.03991v2.pdf</t>
+  </si>
+  <si>
+    <t>https://assemblage-dataset.net/</t>
+  </si>
+  <si>
+    <t>http://doi.acm.org/10.1145/2666652.2666663</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3564625.3567975</t>
+  </si>
+  <si>
+    <t>https://www.usenix.org/conference/usenixsecurity16/technical-sessions/presentation/andriesse</t>
+  </si>
+  <si>
+    <t>https://www.usenix.org/conference/usenixsecurity14/technical-sessions/presentation/bao</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3379597.3387481</t>
+  </si>
+  <si>
+    <t>https://proceedings.neurips.cc/paper_files/paper/2020/file/1457c0d6bfcb4967418bfb8ac142f64a-Paper.pdf</t>
+  </si>
+  <si>
+    <t>https://www.usenix.org/conference/usenixsecurity22/presentation/chen-qibin</t>
+  </si>
+  <si>
+    <t>http://arxiv.org/abs/2205.11794</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3428293</t>
+  </si>
+  <si>
+    <t>https://api.semanticscholar.org/CorpusID:52967399</t>
+  </si>
+  <si>
+    <t>http://arxiv.org/abs/1806.04773</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S0167739X21002090</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3545948.3545956</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.48550/arXiv.2405.03478</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3548606.3560612</t>
+  </si>
+  <si>
+    <t>https://github.com/boozallen/MOTIF</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3605764.3623907</t>
+  </si>
+  <si>
+    <t>http://dx.doi.org/10.1109/TSE.2022.3187689</t>
+  </si>
+  <si>
+    <t>https://github.com/huzecong/ghcc</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S0167404821001954</t>
+  </si>
+  <si>
+    <t>https://api.semanticscholar.org/CorpusID:232134887</t>
+  </si>
+  <si>
+    <t>https://proceedings.mlr.press/v97/li19d.html</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2079-9292/12/7/1722</t>
+  </si>
+  <si>
+    <t>https://www.usenix.org/conference/usenixsecurity22/presentation/marcelli</t>
+  </si>
+  <si>
+    <t>https://vcpkg.io/en/</t>
+  </si>
+  <si>
+    <t>https://api.semanticscholar.org/CorpusID:257532815</t>
+  </si>
+  <si>
+    <t>https://ceur-ws.org/Vol-3652/paper12.pdf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3427228.3427265</t>
+  </si>
+  <si>
+    <t>http://arxiv.org/abs/1909.06674</t>
+  </si>
+  <si>
+    <t>http://arxiv.org/abs/2012.09932</t>
+  </si>
+  <si>
+    <t>http://arxiv.org/abs/2006.09271</t>
+  </si>
+  <si>
+    <t>http://arxiv.org/abs/2009.03779</t>
+  </si>
+  <si>
+    <t>https://virusshare.com/</t>
+  </si>
+  <si>
+    <t>https://www.usenix.org/conference/raid2020/presentation/omar</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3465361</t>
+  </si>
+  <si>
+    <t>http://dx.doi.org/10.1145/3366423.3380145</t>
+  </si>
+  <si>
+    <t>https://api.semanticscholar.org/CorpusID:33377904</t>
+  </si>
+  <si>
+    <t>https://gs.statcounter.com/os-market-share/desktop/worldwide/</t>
+  </si>
+  <si>
+    <t>https://api.semanticscholar.org/CorpusID:249062999</t>
+  </si>
+  <si>
+    <t>https://api.semanticscholar.org/CorpusID:249674500</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/978-3-031-43412-9_16</t>
+  </si>
+  <si>
+    <t>https://www.usenix.org/conference/usenixsecurity22/presentation/yu-sheng</t>
+  </si>
+  <si>
+    <t>https://www.usenix.org/conference/usenixsecurity20/presentation/zhu</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3372297.3420013</t>
+  </si>
+  <si>
+    <t>https://assemblagedocs.readthedocs.io</t>
+  </si>
+  <si>
+    <t>Documentación</t>
+  </si>
+  <si>
+    <t>https://github.com/Assemblage-Dataset/Assemblage</t>
+  </si>
+  <si>
+    <t>https://github.com/Cisco-Talos/binary_function_similarity/</t>
+  </si>
+  <si>
+    <t>2106.04463v3.pdf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7303/syn26376615</t>
+  </si>
+  <si>
+    <t>https://endocv2021.grand-challenge.org</t>
+  </si>
+  <si>
+    <t>https://www.synapse.org/</t>
+  </si>
+  <si>
+    <t>https://www.synapse.org/#!Synapse:syn45200214</t>
+  </si>
+  <si>
+    <t>https://github.com/sharibox/EndoCV2021-polyp_det_seg_gen</t>
+  </si>
+  <si>
+    <t>https://github.com/sharibox/PolypGen-Benchmark.git</t>
+  </si>
+  <si>
+    <t>https://labelbox.com</t>
+  </si>
+  <si>
+    <t>http://www.endoatlas.org/index.php?page=home</t>
+  </si>
+  <si>
+    <t>http://www.pascal-network.org/challenges/VOC/voc2012/workshop/index.html</t>
+  </si>
+  <si>
+    <t>2004.03597v2.pdf</t>
+  </si>
+  <si>
+    <t>http://www.crowd-counting.com</t>
+  </si>
+  <si>
+    <t>1706.08612v2.pdf</t>
+  </si>
+  <si>
+    <t>http://www.robots.ox.ac.uk/~vgg/data/voxceleb</t>
+  </si>
+  <si>
+    <t>http://databases.forensic-voice-comparison.net</t>
+  </si>
+  <si>
+    <t>https://www.sama.com/sama-coco-dataset/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -715,6 +919,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -762,7 +972,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -788,6 +998,18 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -808,9 +1030,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -848,7 +1070,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -954,7 +1176,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1096,7 +1318,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1104,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CACB1099-50E5-47B9-8BC3-1C37A1BD5CEA}">
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E243"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.140625" customWidth="1"/>
@@ -4188,6 +4410,1060 @@
         <v>7</v>
       </c>
       <c r="E181" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5">
+      <c r="A182" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B182" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="C182" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E182" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5">
+      <c r="A183" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B183" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="C183" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D183" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E183" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5">
+      <c r="A184" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B184" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="C184" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D184" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E184" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" ht="30">
+      <c r="A185" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B185" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="C185" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D185" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E185" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" ht="30">
+      <c r="A186" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B186" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="C186" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D186" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E186" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5">
+      <c r="A187" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B187" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="C187" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D187" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E187" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" ht="30">
+      <c r="A188" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B188" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="C188" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D188" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E188" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" ht="30">
+      <c r="A189" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B189" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="C189" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D189" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E189" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5">
+      <c r="A190" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B190" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="C190" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D190" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E190" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5">
+      <c r="A191" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B191" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="C191" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D191" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E191" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5">
+      <c r="A192" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B192" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="C192" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D192" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E192" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5">
+      <c r="A193" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B193" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="C193" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D193" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E193" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" ht="30">
+      <c r="A194" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B194" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="C194" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D194" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E194" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5">
+      <c r="A195" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B195" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="C195" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D195" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E195" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5">
+      <c r="A196" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B196" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="C196" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D196" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E196" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5">
+      <c r="A197" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B197" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C197" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D197" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E197" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5">
+      <c r="A198" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B198" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C198" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D198" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E198" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5">
+      <c r="A199" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B199" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="C199" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D199" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E199" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5">
+      <c r="A200" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B200" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="C200" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D200" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E200" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5">
+      <c r="A201" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B201" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="C201" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D201" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E201" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" ht="30">
+      <c r="A202" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B202" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="C202" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D202" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E202" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5">
+      <c r="A203" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B203" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="C203" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D203" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E203" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5">
+      <c r="A204" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B204" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="C204" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D204" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E204" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5">
+      <c r="A205" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B205" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="C205" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D205" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E205" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" ht="30">
+      <c r="A206" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B206" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="C206" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D206" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E206" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5">
+      <c r="A207" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B207" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="C207" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D207" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E207" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5">
+      <c r="A208" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B208" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="C208" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D208" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E208" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5">
+      <c r="A209" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B209" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="C209" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D209" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E209" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5">
+      <c r="A210" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B210" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="C210" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D210" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E210" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5">
+      <c r="A211" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B211" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="C211" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D211" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E211" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5">
+      <c r="A212" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B212" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="C212" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D212" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E212" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5">
+      <c r="A213" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B213" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="C213" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D213" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E213" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5">
+      <c r="A214" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B214" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="C214" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D214" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E214" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5">
+      <c r="A215" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B215" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C215" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D215" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E215" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5">
+      <c r="A216" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B216" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="C216" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D216" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E216" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5">
+      <c r="A217" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B217" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="C217" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D217" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E217" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5">
+      <c r="A218" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B218" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="C218" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D218" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E218" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5">
+      <c r="A219" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B219" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="C219" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D219" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E219" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" ht="30">
+      <c r="A220" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B220" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="C220" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D220" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E220" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5">
+      <c r="A221" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B221" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="C221" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D221" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E221" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5">
+      <c r="A222" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B222" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="C222" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D222" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E222" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5">
+      <c r="A223" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B223" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="C223" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D223" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E223" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" ht="30">
+      <c r="A224" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B224" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="C224" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D224" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E224" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" ht="30">
+      <c r="A225" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B225" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="C225" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D225" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E225" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5">
+      <c r="A226" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B226" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="C226" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D226" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E226" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5">
+      <c r="A227" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B227" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="C227" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D227" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E227" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5">
+      <c r="A228" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B228" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C228" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D228" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E228" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5">
+      <c r="A229" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B229" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="C229" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D229" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E229" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5">
+      <c r="A230" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B230" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="C230" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D230" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E230" s="13" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5">
+      <c r="A231" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B231" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="C231" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D231" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E231" s="13" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5">
+      <c r="A232" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B232" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="C232" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D232" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E232" s="13" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5">
+      <c r="A233" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B233" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="C233" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D233" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E233" s="13" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5">
+      <c r="A234" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B234" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="C234" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D234" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E234" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5">
+      <c r="A235" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B235" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="C235" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D235" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E235" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5">
+      <c r="A236" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B236" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="C236" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D236" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E236" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5">
+      <c r="A237" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B237" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="C237" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D237" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E237" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" ht="30">
+      <c r="A238" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B238" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="C238" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D238" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E238" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5">
+      <c r="A239" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="B239" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="C239" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D239" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E239" s="13" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5">
+      <c r="A240" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="B240" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="C240" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D240" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E240" s="13" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5">
+      <c r="A241" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="B241" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="C241" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D241" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E241" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5">
+      <c r="A242" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="B242" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="C242" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D242" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E242" s="13" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5">
+      <c r="A243" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="B243" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="C243" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D243" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E243" s="11" t="s">
         <v>210</v>
       </c>
     </row>
@@ -4205,6 +5481,12 @@
     <hyperlink ref="B150" r:id="rId10" xr:uid="{17FADDB5-B760-49FD-89F8-03C950BBE937}"/>
     <hyperlink ref="B156" r:id="rId11" xr:uid="{D19B3E6F-24CE-49C2-95C1-1009E6D365FB}"/>
     <hyperlink ref="B158" r:id="rId12" xr:uid="{8E011266-9DF2-400B-9141-1023DA736D87}"/>
+    <hyperlink ref="B182" r:id="rId13" xr:uid="{4051D2CB-A568-4A46-9BF3-A97636CE2B5F}"/>
+    <hyperlink ref="B228" r:id="rId14" xr:uid="{A42DB6F5-A114-4A93-98C1-8B8F8C248A21}"/>
+    <hyperlink ref="B230" r:id="rId15" xr:uid="{68567B8C-A624-4225-9626-D995C85B9F6A}"/>
+    <hyperlink ref="B231" r:id="rId16" xr:uid="{4581FD07-13C0-4B48-986D-2A626684D4CD}"/>
+    <hyperlink ref="B239" r:id="rId17" xr:uid="{011BB97C-5AD8-4038-8DCF-DB551E7ED7F9}"/>
+    <hyperlink ref="B240" r:id="rId18" xr:uid="{990F102A-4248-4013-86E4-3145D2D14FF6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>